<commit_message>
Bug fixed and additonal reuirments
</commit_message>
<xml_diff>
--- a/output/kpi_summary.xlsx
+++ b/output/kpi_summary.xlsx
@@ -448,15 +448,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,12 +483,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Trend / Note</t>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
         </is>
       </c>
     </row>
@@ -512,12 +518,19 @@
           <t>&lt;= 5.00</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="n">
+        <v>1.3415</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>AMBER</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Slightly above tolerance</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -540,12 +553,19 @@
           <t>&gt;= 95.0%</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Late receipts from Supplier A &amp; Supplier C reduced on-time performance</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -568,12 +588,19 @@
           <t>&lt;= 2.0%</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>0.0576</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Mismatch volume is concentrated with Supplier A &amp; Supplier C</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -591,12 +618,16 @@
           <t>26,454</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Inbound volume processed in the selected period</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -614,12 +645,16 @@
           <t>123</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Late receipts concentrated across Supplier A &amp; Supplier C</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -637,12 +672,12 @@
           <t>Supplier A (9,900), Supplier C (9,630), Supplier B (9,149)</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Ranked by late ordered quantity in the selected period.</t>
         </is>
@@ -669,12 +704,19 @@
           <t>&gt;= 95.0%</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>-0.1287</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>MN-5544 backorders impacted fill rate</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -697,12 +739,19 @@
           <t>&gt;= 92.0%</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>-0.8662</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Late shipments on SO20092 &amp; SO20124</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -725,12 +774,19 @@
           <t>&lt;= 3.0%</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>0.1487</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Backorders concentrated in MN-5544 &amp; BR-2208</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -748,12 +804,16 @@
           <t>1,747</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Outbound volume shipped in the selected period</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -771,12 +831,16 @@
           <t>55</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Late shipments include SO20092 &amp; SO20124</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -794,12 +858,12 @@
           <t>MN-5544 (91), BR-2208 (85), CL-7781 (73), ZX-9910 (70), AX-4312 (61)</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Ranked by backordered quantity in the selected period.</t>
         </is>
@@ -826,12 +890,19 @@
           <t>20.0 to 45.0</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" t="n">
+        <v>14.2581</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Healthy for BR-2208</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -854,12 +925,19 @@
           <t>&lt;= 2.0%</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>0.5123</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CL-7781 stock-out risk at WH-02</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -882,12 +960,19 @@
           <t>&gt;= 95.0%</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>-0.3452</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CL-7781 is below safety stock at WH-02</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -910,12 +995,19 @@
           <t>&lt;= 15.0%</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>0.3661</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Above tolerance</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -933,12 +1025,16 @@
           <t>175.5 days</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Average inventory age across the selected scope</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -956,12 +1052,12 @@
           <t>79.90</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Proxy uses annualized shipped quantity over average on-hand quantity because finance valuation fields are not present.</t>
         </is>
@@ -983,12 +1079,12 @@
           <t>17,754</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Proxy uses aged on-hand quantity because unit_cost is not present in the current data model.</t>
         </is>
@@ -1015,12 +1111,19 @@
           <t>&gt;= 14.00</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>-6.6616</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>WH-03 Night shift throughput is below plan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1043,12 +1146,19 @@
           <t>&gt;= 1.20</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>-0.2261</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>WH-03 Night shift order flow is below plan</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1066,12 +1176,16 @@
           <t>1422.35</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Average daily order volume processed</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1094,12 +1208,19 @@
           <t>&gt;= 95.0%</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>-0.1065</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>WH-03 Night shift missed SLA commitments</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1122,12 +1243,19 @@
           <t>75.0% to 90.0%</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" t="n">
+        <v>-0.0027</v>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Equipment utilization at WH-03 averaged 79.9%</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1150,12 +1278,19 @@
           <t>&lt;= 3.50</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" t="n">
+        <v>-0.0105</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Within tolerance</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1178,12 +1313,19 @@
           <t>&gt;= 14.00</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" t="n">
+        <v>-0.4211</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>AMBER</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Slightly below target</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1206,12 +1348,19 @@
           <t>&lt;= 1.0%</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>AMBER</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Day shift errors from E-1107</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1234,12 +1383,19 @@
           <t>&lt;= 1.5%</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" t="n">
+        <v>-0.0069</v>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Within tolerance</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1262,12 +1418,19 @@
           <t>&lt;= 8.0%</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>0.0956</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Day shift overtime is highest for E-1068</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1285,12 +1448,16 @@
           <t>125</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Average task load per employee record</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1377,7 +1544,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Inbound timeliness is critically low at 0.0%, raising supplier receipt risk.</t>
+          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1424,7 +1591,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Inbound timeliness is critically low at 0.0%, raising supplier receipt risk.</t>
+          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1471,7 +1638,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Inbound timeliness is critically low at 0.0%, raising supplier receipt risk.</t>
+          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1518,7 +1685,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Inbound timeliness is critically low at 0.0%, raising supplier receipt risk.</t>
+          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1560,7 +1727,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Inbound timeliness is critically low at 0.0%, raising supplier receipt risk.</t>
+          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1602,7 +1769,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Inbound timeliness is critically low at 0.0%, raising supplier receipt risk.</t>
+          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1644,7 +1811,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Outbound service is severely impacted with OTIF at 5.4% and backorder rate at 17.9%.</t>
+          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1691,7 +1858,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Outbound service is severely impacted with OTIF at 5.4% and backorder rate at 17.9%.</t>
+          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1738,7 +1905,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Outbound service is severely impacted with OTIF at 5.4% and backorder rate at 17.9%.</t>
+          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1785,7 +1952,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Outbound service is severely impacted with OTIF at 5.4% and backorder rate at 17.9%.</t>
+          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1827,7 +1994,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Outbound service is severely impacted with OTIF at 5.4% and backorder rate at 17.9%.</t>
+          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1869,7 +2036,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Outbound service is severely impacted with OTIF at 5.4% and backorder rate at 17.9%.</t>
+          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1911,7 +2078,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Inventory risk is high with stockout exposure at 53.2% and aged inventory over 51%.</t>
+          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1958,7 +2125,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Inventory risk is high with stockout exposure at 53.2% and aged inventory over 51%.</t>
+          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2005,7 +2172,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Inventory risk is high with stockout exposure at 53.2% and aged inventory over 51%.</t>
+          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2052,7 +2219,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Inventory risk is high with stockout exposure at 53.2% and aged inventory over 51%.</t>
+          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2099,7 +2266,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Inventory risk is high with stockout exposure at 53.2% and aged inventory over 51%.</t>
+          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2141,7 +2308,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Inventory risk is high with stockout exposure at 53.2% and aged inventory over 51%.</t>
+          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2183,7 +2350,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Inventory risk is high with stockout exposure at 53.2% and aged inventory over 51%.</t>
+          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2225,7 +2392,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Warehouse throughput is below target with low lines and orders per labor-hour and SLA adherence at 84.4%.</t>
+          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2272,7 +2439,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Warehouse throughput is below target with low lines and orders per labor-hour and SLA adherence at 84.4%.</t>
+          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2319,7 +2486,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Warehouse throughput is below target with low lines and orders per labor-hour and SLA adherence at 84.4%.</t>
+          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2361,7 +2528,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Warehouse throughput is below target with low lines and orders per labor-hour and SLA adherence at 84.4%.</t>
+          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2408,7 +2575,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Warehouse throughput is below target with low lines and orders per labor-hour and SLA adherence at 84.4%.</t>
+          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2455,7 +2622,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Warehouse throughput is below target with low lines and orders per labor-hour and SLA adherence at 84.4%.</t>
+          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2502,7 +2669,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Workforce efficiency is pressured, shown by high overtime at 17.6% and elevated error rate at 1.6%.</t>
+          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2549,7 +2716,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Workforce efficiency is pressured, shown by high overtime at 17.6% and elevated error rate at 1.6%.</t>
+          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2596,7 +2763,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Workforce efficiency is pressured, shown by high overtime at 17.6% and elevated error rate at 1.6%.</t>
+          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2643,7 +2810,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Workforce efficiency is pressured, shown by high overtime at 17.6% and elevated error rate at 1.6%.</t>
+          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2690,7 +2857,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Workforce efficiency is pressured, shown by high overtime at 17.6% and elevated error rate at 1.6%.</t>
+          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2757,7 +2924,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Inbound receipts on-time are at 0.0%, far below the 95% target.</t>
+          <t>Inbound: Supplier A &amp; Supplier C delays and discrepancies reduced on-time receipts to 0%.</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2936,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Outbound fill rate is 82.1%, missing the 95% goal.</t>
+          <t>Outbound: MN-5544 backorders at 17.9% lowered fill rate to 82.1%, below 95% target.</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2948,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Stockout exposure at 53.2% greatly exceeds the 2% target.</t>
+          <t>Inventory: CL-7781 stock-out exposure at 53.2% and safety stock coverage at 60.5% at WH-02 are critical.</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2960,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lines picked per labor-hour are 7.34, under the 14.0 minimum.</t>
+          <t>Warehouse Productivity: WH-03 Night shift lines picked per labor-hour at 7.34 is half the 14.0 target.</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2972,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Overtime usage is more than double the 8% threshold.</t>
+          <t>Employee Productivity: Day shift error rate at 1.6% exceeds 1.0% target, driven by E-1107.</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2996,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Inventory coverage gaps may continue to drive stockouts and service degradation.</t>
+          <t>Elevated backorders create immediate customer-service and fulfillment risk.</t>
         </is>
       </c>
     </row>
@@ -2841,7 +3008,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Elevated backorders create immediate customer-service and fulfillment risk.</t>
+          <t>Inventory coverage gaps may continue to drive stockouts and service degradation.</t>
         </is>
       </c>
     </row>
@@ -2853,7 +3020,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Prioritize improving supplier on-time receipts to reduce inbound delays.</t>
+          <t>Inbound: Engage Supplier A &amp; Supplier C to reduce late receipts and quantity mismatches.</t>
         </is>
       </c>
     </row>
@@ -2865,7 +3032,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Address outbound backorders to improve fill rate and OTIF performance.</t>
+          <t>Outbound: Prioritize fulfillment and replenishment for MN-5544 to reduce backorders.</t>
         </is>
       </c>
     </row>
@@ -2877,7 +3044,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mitigate inventory risks by reducing stockout exposure and aged inventory.</t>
+          <t>Inventory: Expedite or rebalance stock for CL-7781 at WH-02 to mitigate stock-out risk.</t>
         </is>
       </c>
     </row>
@@ -2889,7 +3056,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Enhance warehouse labor productivity to meet lines and orders per labor-hour targets.</t>
+          <t>Warehouse Productivity: Rebalance labor or adjust maintenance on WH-03 Night shift to improve throughput and SLA adherence.</t>
         </is>
       </c>
     </row>
@@ -2901,7 +3068,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Manage workforce overtime and error rates to improve employee productivity.</t>
+          <t>Employee Productivity: Provide coaching or staffing support for E-1107 and manage overtime for E-1068.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
removed some files and added original reuirment docs
</commit_message>
<xml_diff>
--- a/output/kpi_summary.xlsx
+++ b/output/kpi_summary.xlsx
@@ -1544,7 +1544,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
+          <t>Late receipts from Supplier A &amp; Supplier C reduced on-time performance; engage supplier recovery on delayed receipts.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
+          <t>Late receipts from Supplier A &amp; Supplier C reduced on-time performance; engage supplier recovery on delayed receipts.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
+          <t>Late receipts from Supplier A &amp; Supplier C reduced on-time performance; engage supplier recovery on delayed receipts.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
+          <t>Late receipts from Supplier A &amp; Supplier C reduced on-time performance; engage supplier recovery on delayed receipts.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
+          <t>Late receipts from Supplier A &amp; Supplier C reduced on-time performance; engage supplier recovery on delayed receipts.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Late receipts and quantity discrepancies from Supplier A &amp; Supplier C caused inbound performance failures.</t>
+          <t>Late receipts from Supplier A &amp; Supplier C reduced on-time performance; engage supplier recovery on delayed receipts.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
+          <t>MN-5544 backorders impacted fill rate; review fulfillment and replenishment priorities.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
+          <t>MN-5544 backorders impacted fill rate; review fulfillment and replenishment priorities.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
+          <t>MN-5544 backorders impacted fill rate; review fulfillment and replenishment priorities.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
+          <t>MN-5544 backorders impacted fill rate; review fulfillment and replenishment priorities.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
+          <t>MN-5544 backorders impacted fill rate; review fulfillment and replenishment priorities.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Backorders on MN-5544 and late shipments on SO20092 &amp; SO20124 severely impacted outbound fill rate and OTIF.</t>
+          <t>MN-5544 backorders impacted fill rate; review fulfillment and replenishment priorities.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
+          <t>CL-7781 stock-out risk at WH-02; trigger targeted expedite or stock rebalance.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
+          <t>CL-7781 stock-out risk at WH-02; trigger targeted expedite or stock rebalance.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
+          <t>CL-7781 stock-out risk at WH-02; trigger targeted expedite or stock rebalance.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
+          <t>CL-7781 stock-out risk at WH-02; trigger targeted expedite or stock rebalance.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
+          <t>CL-7781 stock-out risk at WH-02; trigger targeted expedite or stock rebalance.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
+          <t>CL-7781 stock-out risk at WH-02; trigger targeted expedite or stock rebalance.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CL-7781 at WH-02 faces critical stock-out risk with low safety stock coverage and high aged inventory.</t>
+          <t>CL-7781 stock-out risk at WH-02; trigger targeted expedite or stock rebalance.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
+          <t>WH-03 Night shift throughput is below plan; rebalance labor or maintenance windows.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
+          <t>WH-03 Night shift throughput is below plan; rebalance labor or maintenance windows.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
+          <t>WH-03 Night shift throughput is below plan; rebalance labor or maintenance windows.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
+          <t>WH-03 Night shift throughput is below plan; rebalance labor or maintenance windows.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
+          <t>WH-03 Night shift throughput is below plan; rebalance labor or maintenance windows.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>WH-03 Night shift underperforms on throughput and SLA adherence despite adequate equipment utilization.</t>
+          <t>WH-03 Night shift throughput is below plan; rebalance labor or maintenance windows.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
+          <t>Day shift errors from E-1107; add shift-level coaching or staffing support.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
+          <t>Day shift errors from E-1107; add shift-level coaching or staffing support.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
+          <t>Day shift errors from E-1107; add shift-level coaching or staffing support.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
+          <t>Day shift errors from E-1107; add shift-level coaching or staffing support.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Day shift errors from employee E-1107 and high overtime for E-1068 indicate staffing and quality issues.</t>
+          <t>Day shift errors from E-1107; add shift-level coaching or staffing support.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Inbound: Supplier A &amp; Supplier C delays and discrepancies reduced on-time receipts to 0%.</t>
+          <t>Inbound: Late receipts from Supplier A &amp; Supplier C reduced on-time performance; engage supplier capacity or recovery planning.</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Outbound: MN-5544 backorders at 17.9% lowered fill rate to 82.1%, below 95% target.</t>
+          <t>Outbound: MN-5544 backorders impacted fill rate; review safety stock and order-priority settings.</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Inventory: CL-7781 stock-out exposure at 53.2% and safety stock coverage at 60.5% at WH-02 are critical.</t>
+          <t>Inventory: CL-7781 stock-out risk at WH-02; trigger expedite or rebalance inventory.</t>
         </is>
       </c>
     </row>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Warehouse Productivity: WH-03 Night shift lines picked per labor-hour at 7.34 is half the 14.0 target.</t>
+          <t>Warehouse Productivity: WH-03 Night shift throughput is below plan; rebalance labor or maintenance windows.</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Employee Productivity: Day shift error rate at 1.6% exceeds 1.0% target, driven by E-1107.</t>
+          <t>Employee: Day shift errors from E-1107; add refresher training or staffing support.</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Inbound: Engage Supplier A &amp; Supplier C to reduce late receipts and quantity mismatches.</t>
+          <t>Escalate late suppliers and expedite open receipt lines tied to service-risk parts.</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Outbound: Prioritize fulfillment and replenishment for MN-5544 to reduce backorders.</t>
+          <t>Prioritize the SKUs driving backorders and clear the most delayed customer orders first.</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Inventory: Expedite or rebalance stock for CL-7781 at WH-02 to mitigate stock-out risk.</t>
+          <t>Recalibrate reorder points and safety stock for the highest-risk SKUs and constrained warehouses.</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Warehouse Productivity: Rebalance labor or adjust maintenance on WH-03 Night shift to improve throughput and SLA adherence.</t>
+          <t>Address the weakest warehouse throughput driver before adding broader process redesign.</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3068,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Employee Productivity: Provide coaching or staffing support for E-1107 and manage overtime for E-1068.</t>
+          <t>Target the highest-error shift or employee cluster with training and overtime relief.</t>
         </is>
       </c>
     </row>

</xml_diff>